<commit_message>
Revert "Merge branch 'main' of https://github.com/zetdcHre/beii_v1"
This reverts commit a86f0f1d750548858ea6542ba9e0b88dd1c1d59c, reversing
changes made to 2d3cf09acc53b80a8aea1a54770d2673c8adb528.
</commit_message>
<xml_diff>
--- a/budget (1).xlsx
+++ b/budget (1).xlsx
@@ -964,10 +964,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1298,7 +1297,7 @@
     <col min="4" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -1326,7 +1325,7 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -1358,7 +1357,7 @@
       <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2">
         <v>2024</v>
       </c>
       <c r="J2" t="s">
@@ -1390,7 +1389,7 @@
       <c r="H3">
         <v>0</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3">
         <v>2024</v>
       </c>
       <c r="J3" t="s">
@@ -1422,7 +1421,7 @@
       <c r="H4">
         <v>0</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4">
         <v>2024</v>
       </c>
       <c r="J4" t="s">
@@ -1454,7 +1453,7 @@
       <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5">
         <v>2024</v>
       </c>
       <c r="J5" t="s">
@@ -1486,7 +1485,7 @@
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6">
         <v>2024</v>
       </c>
       <c r="J6" t="s">
@@ -1518,7 +1517,7 @@
       <c r="H7">
         <v>0</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7">
         <v>2024</v>
       </c>
       <c r="J7" t="s">
@@ -1550,7 +1549,7 @@
       <c r="H8">
         <v>0</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8">
         <v>2024</v>
       </c>
       <c r="J8" t="s">
@@ -1582,7 +1581,7 @@
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9">
         <v>2024</v>
       </c>
       <c r="J9" t="s">
@@ -1614,7 +1613,7 @@
       <c r="H10">
         <v>0</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10">
         <v>2024</v>
       </c>
       <c r="J10" t="s">
@@ -1646,7 +1645,7 @@
       <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11">
         <v>2024</v>
       </c>
       <c r="J11" t="s">
@@ -1678,7 +1677,7 @@
       <c r="H12">
         <v>0</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12">
         <v>2024</v>
       </c>
       <c r="J12" t="s">
@@ -1710,7 +1709,7 @@
       <c r="H13">
         <v>0</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13">
         <v>2024</v>
       </c>
       <c r="J13" t="s">
@@ -1742,7 +1741,7 @@
       <c r="H14">
         <v>0</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14">
         <v>2024</v>
       </c>
       <c r="J14" t="s">
@@ -1774,7 +1773,7 @@
       <c r="H15">
         <v>0</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15">
         <v>2024</v>
       </c>
       <c r="J15" t="s">
@@ -1806,7 +1805,7 @@
       <c r="H16">
         <v>0</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16">
         <v>2024</v>
       </c>
       <c r="J16" t="s">
@@ -1838,7 +1837,7 @@
       <c r="H17">
         <v>0</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17">
         <v>2024</v>
       </c>
       <c r="J17" t="s">
@@ -1870,7 +1869,7 @@
       <c r="H18">
         <v>0</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18">
         <v>2024</v>
       </c>
       <c r="J18" t="s">
@@ -1902,7 +1901,7 @@
       <c r="H19">
         <v>0</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19">
         <v>2024</v>
       </c>
       <c r="J19" t="s">
@@ -1934,7 +1933,7 @@
       <c r="H20">
         <v>0</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20">
         <v>2024</v>
       </c>
       <c r="J20" t="s">
@@ -1966,7 +1965,7 @@
       <c r="H21">
         <v>0</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21">
         <v>2024</v>
       </c>
       <c r="J21" t="s">
@@ -1998,7 +1997,7 @@
       <c r="H22">
         <v>0</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22">
         <v>2024</v>
       </c>
       <c r="J22" t="s">
@@ -2030,7 +2029,7 @@
       <c r="H23">
         <v>0</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23">
         <v>2024</v>
       </c>
       <c r="J23" t="s">
@@ -2062,7 +2061,7 @@
       <c r="H24">
         <v>0</v>
       </c>
-      <c r="I24" s="2">
+      <c r="I24">
         <v>2024</v>
       </c>
       <c r="J24" t="s">
@@ -2094,7 +2093,7 @@
       <c r="H25">
         <v>1500000</v>
       </c>
-      <c r="I25" s="2">
+      <c r="I25">
         <v>2024</v>
       </c>
       <c r="J25" t="s">
@@ -2126,7 +2125,7 @@
       <c r="H26">
         <v>0</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26">
         <v>2024</v>
       </c>
       <c r="J26" t="s">
@@ -2158,7 +2157,7 @@
       <c r="H27">
         <v>0</v>
       </c>
-      <c r="I27" s="2">
+      <c r="I27">
         <v>2024</v>
       </c>
       <c r="J27" t="s">
@@ -2190,7 +2189,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="I28" s="2">
+      <c r="I28">
         <v>2024</v>
       </c>
       <c r="J28" t="s">
@@ -2222,7 +2221,7 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="I29" s="2">
+      <c r="I29">
         <v>2024</v>
       </c>
       <c r="J29" t="s">
@@ -2254,7 +2253,7 @@
       <c r="H30">
         <v>0</v>
       </c>
-      <c r="I30" s="2">
+      <c r="I30">
         <v>2024</v>
       </c>
       <c r="J30" t="s">
@@ -2286,7 +2285,7 @@
       <c r="H31">
         <v>0</v>
       </c>
-      <c r="I31" s="2">
+      <c r="I31">
         <v>2024</v>
       </c>
       <c r="J31" t="s">
@@ -2318,7 +2317,7 @@
       <c r="H32">
         <v>0</v>
       </c>
-      <c r="I32" s="2">
+      <c r="I32">
         <v>2024</v>
       </c>
       <c r="J32" t="s">
@@ -2350,7 +2349,7 @@
       <c r="H33">
         <v>0</v>
       </c>
-      <c r="I33" s="2">
+      <c r="I33">
         <v>2024</v>
       </c>
       <c r="J33" t="s">
@@ -2382,7 +2381,7 @@
       <c r="H34">
         <v>0</v>
       </c>
-      <c r="I34" s="2">
+      <c r="I34">
         <v>2024</v>
       </c>
       <c r="J34" t="s">
@@ -2414,7 +2413,7 @@
       <c r="H35">
         <v>0</v>
       </c>
-      <c r="I35" s="2">
+      <c r="I35">
         <v>2024</v>
       </c>
       <c r="J35" t="s">
@@ -2446,7 +2445,7 @@
       <c r="H36">
         <v>0</v>
       </c>
-      <c r="I36" s="2">
+      <c r="I36">
         <v>2024</v>
       </c>
       <c r="J36" t="s">
@@ -2478,7 +2477,7 @@
       <c r="H37">
         <v>0</v>
       </c>
-      <c r="I37" s="2">
+      <c r="I37">
         <v>2024</v>
       </c>
       <c r="J37" t="s">
@@ -2510,7 +2509,7 @@
       <c r="H38">
         <v>0</v>
       </c>
-      <c r="I38" s="2">
+      <c r="I38">
         <v>2024</v>
       </c>
       <c r="J38" t="s">
@@ -2542,7 +2541,7 @@
       <c r="H39">
         <v>0</v>
       </c>
-      <c r="I39" s="2">
+      <c r="I39">
         <v>2024</v>
       </c>
       <c r="J39" t="s">
@@ -2574,7 +2573,7 @@
       <c r="H40">
         <v>0</v>
       </c>
-      <c r="I40" s="2">
+      <c r="I40">
         <v>2024</v>
       </c>
       <c r="J40" t="s">
@@ -2606,7 +2605,7 @@
       <c r="H41">
         <v>0</v>
       </c>
-      <c r="I41" s="2">
+      <c r="I41">
         <v>2024</v>
       </c>
       <c r="J41" t="s">
@@ -2638,7 +2637,7 @@
       <c r="H42">
         <v>0</v>
       </c>
-      <c r="I42" s="2">
+      <c r="I42">
         <v>2024</v>
       </c>
       <c r="J42" t="s">
@@ -2670,7 +2669,7 @@
       <c r="H43">
         <v>0</v>
       </c>
-      <c r="I43" s="2">
+      <c r="I43">
         <v>2024</v>
       </c>
       <c r="J43" t="s">
@@ -2702,7 +2701,7 @@
       <c r="H44">
         <v>0</v>
       </c>
-      <c r="I44" s="2">
+      <c r="I44">
         <v>2024</v>
       </c>
       <c r="J44" t="s">
@@ -2734,7 +2733,7 @@
       <c r="H45">
         <v>0</v>
       </c>
-      <c r="I45" s="2">
+      <c r="I45">
         <v>2024</v>
       </c>
       <c r="J45" t="s">
@@ -2766,7 +2765,7 @@
       <c r="H46">
         <v>0</v>
       </c>
-      <c r="I46" s="2">
+      <c r="I46">
         <v>2024</v>
       </c>
       <c r="J46" t="s">
@@ -2798,7 +2797,7 @@
       <c r="H47">
         <v>0</v>
       </c>
-      <c r="I47" s="2">
+      <c r="I47">
         <v>2024</v>
       </c>
       <c r="J47" t="s">
@@ -2830,7 +2829,7 @@
       <c r="H48">
         <v>0</v>
       </c>
-      <c r="I48" s="2">
+      <c r="I48">
         <v>2024</v>
       </c>
       <c r="J48" t="s">
@@ -2862,7 +2861,7 @@
       <c r="H49">
         <v>0</v>
       </c>
-      <c r="I49" s="2">
+      <c r="I49">
         <v>2024</v>
       </c>
       <c r="J49" t="s">
@@ -2894,7 +2893,7 @@
       <c r="H50">
         <v>0</v>
       </c>
-      <c r="I50" s="2">
+      <c r="I50">
         <v>2024</v>
       </c>
       <c r="J50" t="s">
@@ -2926,7 +2925,7 @@
       <c r="H51">
         <v>0</v>
       </c>
-      <c r="I51" s="2">
+      <c r="I51">
         <v>2024</v>
       </c>
       <c r="J51" t="s">
@@ -2958,7 +2957,7 @@
       <c r="H52">
         <v>0</v>
       </c>
-      <c r="I52" s="2">
+      <c r="I52">
         <v>2024</v>
       </c>
       <c r="J52" t="s">
@@ -2990,7 +2989,7 @@
       <c r="H53">
         <v>0</v>
       </c>
-      <c r="I53" s="2">
+      <c r="I53">
         <v>2024</v>
       </c>
       <c r="J53" t="s">
@@ -3022,7 +3021,7 @@
       <c r="H54">
         <v>0</v>
       </c>
-      <c r="I54" s="2">
+      <c r="I54">
         <v>2024</v>
       </c>
       <c r="J54" t="s">
@@ -3054,7 +3053,7 @@
       <c r="H55">
         <v>0</v>
       </c>
-      <c r="I55" s="2">
+      <c r="I55">
         <v>2024</v>
       </c>
       <c r="J55" t="s">
@@ -3086,7 +3085,7 @@
       <c r="H56">
         <v>0</v>
       </c>
-      <c r="I56" s="2">
+      <c r="I56">
         <v>2024</v>
       </c>
       <c r="J56" t="s">
@@ -3118,7 +3117,7 @@
       <c r="H57">
         <v>70000000</v>
       </c>
-      <c r="I57" s="2">
+      <c r="I57">
         <v>2024</v>
       </c>
       <c r="J57" t="s">
@@ -3150,7 +3149,7 @@
       <c r="H58">
         <v>0</v>
       </c>
-      <c r="I58" s="2">
+      <c r="I58">
         <v>2024</v>
       </c>
       <c r="J58" t="s">
@@ -3182,7 +3181,7 @@
       <c r="H59">
         <v>0</v>
       </c>
-      <c r="I59" s="2">
+      <c r="I59">
         <v>2024</v>
       </c>
       <c r="J59" t="s">
@@ -3214,7 +3213,7 @@
       <c r="H60">
         <v>0</v>
       </c>
-      <c r="I60" s="2">
+      <c r="I60">
         <v>2024</v>
       </c>
       <c r="J60" t="s">
@@ -3246,7 +3245,7 @@
       <c r="H61">
         <v>0</v>
       </c>
-      <c r="I61" s="2">
+      <c r="I61">
         <v>2024</v>
       </c>
       <c r="J61" t="s">
@@ -3278,7 +3277,7 @@
       <c r="H62">
         <v>0</v>
       </c>
-      <c r="I62" s="2">
+      <c r="I62">
         <v>2024</v>
       </c>
       <c r="J62" t="s">
@@ -3310,7 +3309,7 @@
       <c r="H63">
         <v>109000000</v>
       </c>
-      <c r="I63" s="2">
+      <c r="I63">
         <v>2024</v>
       </c>
       <c r="J63" t="s">
@@ -3342,7 +3341,7 @@
       <c r="H64">
         <v>0</v>
       </c>
-      <c r="I64" s="2">
+      <c r="I64">
         <v>2024</v>
       </c>
       <c r="J64" t="s">
@@ -3374,7 +3373,7 @@
       <c r="H65">
         <v>28000000</v>
       </c>
-      <c r="I65" s="2">
+      <c r="I65">
         <v>2024</v>
       </c>
       <c r="J65" t="s">
@@ -3406,7 +3405,7 @@
       <c r="H66">
         <v>0</v>
       </c>
-      <c r="I66" s="2">
+      <c r="I66">
         <v>2024</v>
       </c>
       <c r="J66" t="s">
@@ -3438,7 +3437,7 @@
       <c r="H67">
         <v>0</v>
       </c>
-      <c r="I67" s="2">
+      <c r="I67">
         <v>2024</v>
       </c>
       <c r="J67" t="s">
@@ -3470,7 +3469,7 @@
       <c r="H68">
         <v>0</v>
       </c>
-      <c r="I68" s="2">
+      <c r="I68">
         <v>2024</v>
       </c>
       <c r="J68" t="s">
@@ -3502,7 +3501,7 @@
       <c r="H69">
         <v>0</v>
       </c>
-      <c r="I69" s="2">
+      <c r="I69">
         <v>2024</v>
       </c>
       <c r="J69" t="s">
@@ -3534,7 +3533,7 @@
       <c r="H70">
         <v>175999999.99000001</v>
       </c>
-      <c r="I70" s="2">
+      <c r="I70">
         <v>2024</v>
       </c>
       <c r="J70" t="s">
@@ -3566,7 +3565,7 @@
       <c r="H71">
         <v>0</v>
       </c>
-      <c r="I71" s="2">
+      <c r="I71">
         <v>2024</v>
       </c>
       <c r="J71" t="s">
@@ -3598,7 +3597,7 @@
       <c r="H72">
         <v>0</v>
       </c>
-      <c r="I72" s="2">
+      <c r="I72">
         <v>2024</v>
       </c>
       <c r="J72" t="s">
@@ -3630,7 +3629,7 @@
       <c r="H73">
         <v>0</v>
       </c>
-      <c r="I73" s="2">
+      <c r="I73">
         <v>2024</v>
       </c>
       <c r="J73" t="s">
@@ -3662,7 +3661,7 @@
       <c r="H74">
         <v>0</v>
       </c>
-      <c r="I74" s="2">
+      <c r="I74">
         <v>2024</v>
       </c>
       <c r="J74" t="s">
@@ -3694,7 +3693,7 @@
       <c r="H75">
         <v>0</v>
       </c>
-      <c r="I75" s="2">
+      <c r="I75">
         <v>2024</v>
       </c>
       <c r="J75" t="s">
@@ -3726,7 +3725,7 @@
       <c r="H76">
         <v>0</v>
       </c>
-      <c r="I76" s="2">
+      <c r="I76">
         <v>2024</v>
       </c>
       <c r="J76" t="s">
@@ -3758,7 +3757,7 @@
       <c r="H77">
         <v>0</v>
       </c>
-      <c r="I77" s="2">
+      <c r="I77">
         <v>2024</v>
       </c>
       <c r="J77" t="s">
@@ -3790,7 +3789,7 @@
       <c r="H78">
         <v>0</v>
       </c>
-      <c r="I78" s="2">
+      <c r="I78">
         <v>2024</v>
       </c>
       <c r="J78" t="s">
@@ -3822,7 +3821,7 @@
       <c r="H79">
         <v>0</v>
       </c>
-      <c r="I79" s="2">
+      <c r="I79">
         <v>2024</v>
       </c>
       <c r="J79" t="s">
@@ -3854,7 +3853,7 @@
       <c r="H80">
         <v>0</v>
       </c>
-      <c r="I80" s="2">
+      <c r="I80">
         <v>2024</v>
       </c>
       <c r="J80" t="s">
@@ -3886,7 +3885,7 @@
       <c r="H81">
         <v>0</v>
       </c>
-      <c r="I81" s="2">
+      <c r="I81">
         <v>2024</v>
       </c>
       <c r="J81" t="s">
@@ -3918,7 +3917,7 @@
       <c r="H82">
         <v>0</v>
       </c>
-      <c r="I82" s="2">
+      <c r="I82">
         <v>2024</v>
       </c>
       <c r="J82" t="s">
@@ -3950,7 +3949,7 @@
       <c r="H83">
         <v>0</v>
       </c>
-      <c r="I83" s="2">
+      <c r="I83">
         <v>2024</v>
       </c>
       <c r="J83" t="s">
@@ -3982,7 +3981,7 @@
       <c r="H84">
         <v>0</v>
       </c>
-      <c r="I84" s="2">
+      <c r="I84">
         <v>2024</v>
       </c>
       <c r="J84" t="s">
@@ -4014,7 +4013,7 @@
       <c r="H85">
         <v>0</v>
       </c>
-      <c r="I85" s="2">
+      <c r="I85">
         <v>2024</v>
       </c>
       <c r="J85" t="s">
@@ -4046,7 +4045,7 @@
       <c r="H86">
         <v>7000000</v>
       </c>
-      <c r="I86" s="2">
+      <c r="I86">
         <v>2024</v>
       </c>
       <c r="J86" t="s">
@@ -4078,7 +4077,7 @@
       <c r="H87">
         <v>0</v>
       </c>
-      <c r="I87" s="2">
+      <c r="I87">
         <v>2024</v>
       </c>
       <c r="J87" t="s">
@@ -4110,7 +4109,7 @@
       <c r="H88">
         <v>0</v>
       </c>
-      <c r="I88" s="2">
+      <c r="I88">
         <v>2024</v>
       </c>
       <c r="J88" t="s">
@@ -4142,7 +4141,7 @@
       <c r="H89">
         <v>0</v>
       </c>
-      <c r="I89" s="2">
+      <c r="I89">
         <v>2024</v>
       </c>
       <c r="J89" t="s">
@@ -4174,7 +4173,7 @@
       <c r="H90">
         <v>0</v>
       </c>
-      <c r="I90" s="2">
+      <c r="I90">
         <v>2024</v>
       </c>
       <c r="J90" t="s">
@@ -4206,7 +4205,7 @@
       <c r="H91">
         <v>0</v>
       </c>
-      <c r="I91" s="2">
+      <c r="I91">
         <v>2024</v>
       </c>
       <c r="J91" t="s">
@@ -4238,7 +4237,7 @@
       <c r="H92">
         <v>0</v>
       </c>
-      <c r="I92" s="2">
+      <c r="I92">
         <v>2024</v>
       </c>
       <c r="J92" t="s">
@@ -4270,7 +4269,7 @@
       <c r="H93">
         <v>0</v>
       </c>
-      <c r="I93" s="2">
+      <c r="I93">
         <v>2024</v>
       </c>
       <c r="J93" t="s">
@@ -4302,7 +4301,7 @@
       <c r="H94">
         <v>40000000</v>
       </c>
-      <c r="I94" s="2">
+      <c r="I94">
         <v>2024</v>
       </c>
       <c r="J94" t="s">
@@ -4334,7 +4333,7 @@
       <c r="H95">
         <v>0</v>
       </c>
-      <c r="I95" s="2">
+      <c r="I95">
         <v>2024</v>
       </c>
       <c r="J95" t="s">
@@ -4366,7 +4365,7 @@
       <c r="H96">
         <v>0</v>
       </c>
-      <c r="I96" s="2">
+      <c r="I96">
         <v>2024</v>
       </c>
       <c r="J96" t="s">
@@ -4398,7 +4397,7 @@
       <c r="H97">
         <v>0</v>
       </c>
-      <c r="I97" s="2">
+      <c r="I97">
         <v>2024</v>
       </c>
       <c r="J97" t="s">
@@ -4430,7 +4429,7 @@
       <c r="H98">
         <v>0</v>
       </c>
-      <c r="I98" s="2">
+      <c r="I98">
         <v>2024</v>
       </c>
       <c r="J98" t="s">
@@ -4462,7 +4461,7 @@
       <c r="H99">
         <v>0</v>
       </c>
-      <c r="I99" s="2">
+      <c r="I99">
         <v>2024</v>
       </c>
       <c r="J99" t="s">
@@ -4494,7 +4493,7 @@
       <c r="H100">
         <v>0</v>
       </c>
-      <c r="I100" s="2">
+      <c r="I100">
         <v>2024</v>
       </c>
       <c r="J100" t="s">
@@ -4526,7 +4525,7 @@
       <c r="H101">
         <v>0</v>
       </c>
-      <c r="I101" s="2">
+      <c r="I101">
         <v>2024</v>
       </c>
       <c r="J101" t="s">
@@ -4558,7 +4557,7 @@
       <c r="H102">
         <v>0</v>
       </c>
-      <c r="I102" s="2">
+      <c r="I102">
         <v>2024</v>
       </c>
       <c r="J102" t="s">
@@ -4590,7 +4589,7 @@
       <c r="H103">
         <v>0</v>
       </c>
-      <c r="I103" s="2">
+      <c r="I103">
         <v>2024</v>
       </c>
       <c r="J103" t="s">
@@ -4622,7 +4621,7 @@
       <c r="H104">
         <v>0</v>
       </c>
-      <c r="I104" s="2">
+      <c r="I104">
         <v>2024</v>
       </c>
       <c r="J104" t="s">
@@ -4654,7 +4653,7 @@
       <c r="H105">
         <v>0</v>
       </c>
-      <c r="I105" s="2">
+      <c r="I105">
         <v>2024</v>
       </c>
       <c r="J105" t="s">
@@ -4686,7 +4685,7 @@
       <c r="H106">
         <v>0</v>
       </c>
-      <c r="I106" s="2">
+      <c r="I106">
         <v>2024</v>
       </c>
       <c r="J106" t="s">
@@ -4718,7 +4717,7 @@
       <c r="H107">
         <v>0</v>
       </c>
-      <c r="I107" s="2">
+      <c r="I107">
         <v>2024</v>
       </c>
       <c r="J107" t="s">
@@ -4750,7 +4749,7 @@
       <c r="H108">
         <v>0</v>
       </c>
-      <c r="I108" s="2">
+      <c r="I108">
         <v>2024</v>
       </c>
       <c r="J108" t="s">
@@ -4782,7 +4781,7 @@
       <c r="H109">
         <v>700000000</v>
       </c>
-      <c r="I109" s="2">
+      <c r="I109">
         <v>2024</v>
       </c>
       <c r="J109" t="s">
@@ -4814,7 +4813,7 @@
       <c r="H110">
         <v>0</v>
       </c>
-      <c r="I110" s="2">
+      <c r="I110">
         <v>2024</v>
       </c>
       <c r="J110" t="s">
@@ -4846,7 +4845,7 @@
       <c r="H111">
         <v>0</v>
       </c>
-      <c r="I111" s="2">
+      <c r="I111">
         <v>2024</v>
       </c>
       <c r="J111" t="s">
@@ -4878,7 +4877,7 @@
       <c r="H112">
         <v>27000000</v>
       </c>
-      <c r="I112" s="2">
+      <c r="I112">
         <v>2024</v>
       </c>
       <c r="J112" t="s">
@@ -4910,7 +4909,7 @@
       <c r="H113">
         <v>0</v>
       </c>
-      <c r="I113" s="2">
+      <c r="I113">
         <v>2024</v>
       </c>
       <c r="J113" t="s">
@@ -4942,7 +4941,7 @@
       <c r="H114">
         <v>0</v>
       </c>
-      <c r="I114" s="2">
+      <c r="I114">
         <v>2024</v>
       </c>
       <c r="J114" t="s">
@@ -4974,7 +4973,7 @@
       <c r="H115">
         <v>0</v>
       </c>
-      <c r="I115" s="2">
+      <c r="I115">
         <v>2024</v>
       </c>
       <c r="J115" t="s">
@@ -5006,7 +5005,7 @@
       <c r="H116">
         <v>0</v>
       </c>
-      <c r="I116" s="2">
+      <c r="I116">
         <v>2024</v>
       </c>
       <c r="J116" t="s">
@@ -5038,7 +5037,7 @@
       <c r="H117">
         <v>0</v>
       </c>
-      <c r="I117" s="2">
+      <c r="I117">
         <v>2024</v>
       </c>
       <c r="J117" t="s">
@@ -5070,7 +5069,7 @@
       <c r="H118">
         <v>5000000</v>
       </c>
-      <c r="I118" s="2">
+      <c r="I118">
         <v>2024</v>
       </c>
       <c r="J118" t="s">
@@ -5102,7 +5101,7 @@
       <c r="H119">
         <v>0</v>
       </c>
-      <c r="I119" s="2">
+      <c r="I119">
         <v>2024</v>
       </c>
       <c r="J119" t="s">
@@ -5134,7 +5133,7 @@
       <c r="H120">
         <v>0</v>
       </c>
-      <c r="I120" s="2">
+      <c r="I120">
         <v>2024</v>
       </c>
       <c r="J120" t="s">
@@ -5166,7 +5165,7 @@
       <c r="H121">
         <v>0</v>
       </c>
-      <c r="I121" s="2">
+      <c r="I121">
         <v>2024</v>
       </c>
       <c r="J121" t="s">
@@ -5198,7 +5197,7 @@
       <c r="H122">
         <v>0</v>
       </c>
-      <c r="I122" s="2">
+      <c r="I122">
         <v>2024</v>
       </c>
       <c r="J122" t="s">
@@ -5230,7 +5229,7 @@
       <c r="H123">
         <v>0</v>
       </c>
-      <c r="I123" s="2">
+      <c r="I123">
         <v>2024</v>
       </c>
       <c r="J123" t="s">
@@ -5262,7 +5261,7 @@
       <c r="H124">
         <v>0</v>
       </c>
-      <c r="I124" s="2">
+      <c r="I124">
         <v>2024</v>
       </c>
       <c r="J124" t="s">
@@ -5294,7 +5293,7 @@
       <c r="H125">
         <v>0</v>
       </c>
-      <c r="I125" s="2">
+      <c r="I125">
         <v>2024</v>
       </c>
       <c r="J125" t="s">
@@ -5326,7 +5325,7 @@
       <c r="H126">
         <v>0</v>
       </c>
-      <c r="I126" s="2">
+      <c r="I126">
         <v>2024</v>
       </c>
       <c r="J126" t="s">
@@ -5358,7 +5357,7 @@
       <c r="H127">
         <v>0</v>
       </c>
-      <c r="I127" s="2">
+      <c r="I127">
         <v>2024</v>
       </c>
       <c r="J127" t="s">
@@ -5390,7 +5389,7 @@
       <c r="H128">
         <v>0</v>
       </c>
-      <c r="I128" s="2">
+      <c r="I128">
         <v>2024</v>
       </c>
       <c r="J128" t="s">
@@ -5422,7 +5421,7 @@
       <c r="H129">
         <v>0</v>
       </c>
-      <c r="I129" s="2">
+      <c r="I129">
         <v>2024</v>
       </c>
       <c r="J129" t="s">
@@ -5454,7 +5453,7 @@
       <c r="H130">
         <v>0</v>
       </c>
-      <c r="I130" s="2">
+      <c r="I130">
         <v>2024</v>
       </c>
       <c r="J130" t="s">
@@ -5486,7 +5485,7 @@
       <c r="H131">
         <v>0</v>
       </c>
-      <c r="I131" s="2">
+      <c r="I131">
         <v>2024</v>
       </c>
       <c r="J131" t="s">
@@ -5495,6 +5494,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>